<commit_message>
[20260310_115400_vd_ingame_masterdata_generation] ブロック基礎設計 vd_osh_boss_00001 xlsx更新
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_osh_boss_00001/vd_osh_boss_00001.xlsx
+++ b/domain/tasks/20260310_115400_vd_ingame_masterdata_generation/vd-ingame-creator/vd_osh_boss_00001/vd_osh_boss_00001.xlsx
@@ -982,7 +982,11 @@
           <t>1コマ</t>
         </is>
       </c>
-      <c r="D14" s="27" t="inlineStr"/>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>osh_00001</t>
+        </is>
+      </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
           <t>None</t>
@@ -990,7 +994,7 @@
       </c>
       <c r="F14" s="27" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -1329,7 +1333,7 @@
       </c>
       <c r="I28" s="27" t="inlineStr">
         <is>
-          <t>雑魚（共通）</t>
+          <t>雑魚（e_キャラ）</t>
         </is>
       </c>
       <c r="J28" s="2" t="n"/>
@@ -1562,7 +1566,7 @@
       </c>
       <c r="H40" s="27" t="inlineStr">
         <is>
-          <t>ボス降臨・summon_position=1.7（ゲート付近）</t>
+          <t>ボス登場・敵ゲート前に降臨（summon_position=1.7）</t>
         </is>
       </c>
       <c r="I40" s="2" t="n"/>
@@ -1599,7 +1603,7 @@
       </c>
       <c r="H41" s="27" t="inlineStr">
         <is>
-          <t>0.5秒後に1体出現・プレッシャー付与</t>
+          <t>ボス登場0.5秒後・プレッシャー</t>
         </is>
       </c>
       <c r="I41" s="2" t="n"/>
@@ -1636,7 +1640,7 @@
       </c>
       <c r="H42" s="27" t="inlineStr">
         <is>
-          <t>3秒後に3体追加・継続的な圧力</t>
+          <t>3秒後・継続的な圧力</t>
         </is>
       </c>
       <c r="I42" s="2" t="n"/>
@@ -1889,7 +1893,7 @@
           <t>バトルヒント</t>
         </is>
       </c>
-      <c r="C58" s="18" t="inlineStr"/>
+      <c r="C58" s="27" t="inlineStr"/>
       <c r="D58" s="28" t="n"/>
       <c r="E58" s="28" t="n"/>
       <c r="F58" s="28" t="n"/>
@@ -1908,7 +1912,7 @@
           <t>ステージ説明文</t>
         </is>
       </c>
-      <c r="C59" s="18" t="inlineStr"/>
+      <c r="C59" s="27" t="inlineStr"/>
       <c r="D59" s="28" t="n"/>
       <c r="E59" s="28" t="n"/>
       <c r="F59" s="28" t="n"/>

</xml_diff>